<commit_message>
Added RDF data schemes and fixed visual schemes for food-table01-06
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/food-table01.xlsx
+++ b/sources/table_normalization/xlsx/food-table01.xlsx
@@ -141,18 +141,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -169,7 +163,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -177,8 +171,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -668,8 +660,8 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3">
@@ -823,8 +815,8 @@
       <c r="A16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="3">

</xml_diff>